<commit_message>
slight add in doc sphinx and test plans
</commit_message>
<xml_diff>
--- a/docs/dqm-ml_test_plan.xlsx
+++ b/docs/dqm-ml_test_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\FONDATION\Support_composants\DQM\dqm-ml\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{D4EED894-366A-4121-B4F9-1DE37F96A6E1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{3B470FB3-6195-4D65-8932-2B985D38052A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19160" windowHeight="7970" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19155" windowHeight="7965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Strategy" sheetId="3" r:id="rId1"/>
@@ -24,23 +24,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="134" uniqueCount="96">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="137" uniqueCount="99">
   <si>
     <t>DQM-ML</t>
   </si>
@@ -700,6 +689,15 @@
   - unrecognized file extension
  -  non homogenous files in folders
 </t>
+  </si>
+  <si>
+    <t>G08</t>
+  </si>
+  <si>
+    <t>Vulnerabilities check</t>
+  </si>
+  <si>
+    <t>CVE ( common vulnerability and exposure)  (on dependencies)</t>
   </si>
 </sst>
 </file>
@@ -753,7 +751,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="27">
     <border>
       <start/>
       <end/>
@@ -1078,11 +1076,42 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <start style="thin">
+        <color indexed="64"/>
+      </start>
+      <end/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <start style="thin">
+        <color indexed="64"/>
+      </start>
+      <end style="thin">
+        <color indexed="64"/>
+      </end>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <start style="thin">
+        <color indexed="64"/>
+      </start>
+      <end style="medium">
+        <color indexed="64"/>
+      </end>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1196,6 +1225,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1510,17 +1542,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E428F4C8-CD47-46B1-8E6D-0591DCDF9390}">
-  <dimension ref="A2:D24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A2:D25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.453125" customWidth="1"/>
-    <col min="2" max="2" width="23.453125" customWidth="1"/>
-    <col min="3" max="3" width="79.453125" customWidth="1"/>
-    <col min="4" max="4" width="33.26953125" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="2" width="23.42578125" customWidth="1"/>
+    <col min="3" max="3" width="79.42578125" customWidth="1"/>
+    <col min="4" max="4" width="33.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
@@ -1532,26 +1564,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="180" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="6"/>
       <c r="C4" s="12" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
       <c r="B5" s="6"/>
       <c r="C5" s="13"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="42"/>
       <c r="C6" s="43"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>5</v>
       </c>
@@ -1562,7 +1594,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>8</v>
       </c>
@@ -1573,7 +1605,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>11</v>
       </c>
@@ -1584,7 +1616,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>14</v>
       </c>
@@ -1595,7 +1627,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>17</v>
       </c>
@@ -1606,7 +1638,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>20</v>
       </c>
@@ -1617,7 +1649,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14" t="s">
         <v>23</v>
       </c>
@@ -1628,95 +1660,107 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="17" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="30" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="56" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="57" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="145" x14ac:dyDescent="0.35">
-      <c r="A15" s="18" t="s">
+    <row r="16" spans="1:4" ht="165" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B16" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C16" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="37" t="s">
+      <c r="D16" s="37" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="18" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B17" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C17" s="12" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="40" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B18" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C18" s="24" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="B18" s="38"/>
-      <c r="C18" s="10"/>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="39" t="s">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="38"/>
+      <c r="C19" s="10"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="39" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="6"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="11" t="s">
+      <c r="B20" s="6"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
         <v>38</v>
-      </c>
-      <c r="B20" s="6"/>
-      <c r="C20" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="11" t="s">
-        <v>40</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="13" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B22" s="6"/>
+      <c r="C22" s="13" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="11" t="s">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="13" t="s">
+      <c r="B23" s="15"/>
+      <c r="C23" s="13" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="14" t="s">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="20"/>
-      <c r="C23" s="16" t="s">
+      <c r="B24" s="20"/>
+      <c r="C24" s="16" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="20"/>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="20"/>
+      <c r="C25" s="55"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1730,22 +1774,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39E4F67D-5E5E-426E-AD85-D031E65C326A}">
   <dimension ref="A1:L36"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.453125" customWidth="1"/>
-    <col min="2" max="2" width="7.1796875" customWidth="1"/>
-    <col min="3" max="3" width="21.26953125" customWidth="1"/>
-    <col min="4" max="4" width="73.26953125" customWidth="1"/>
+    <col min="1" max="1" width="8.42578125" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" customWidth="1"/>
+    <col min="4" max="4" width="73.28515625" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
     <col min="6" max="7" width="23" customWidth="1"/>
-    <col min="8" max="8" width="23.453125" customWidth="1"/>
-    <col min="9" max="9" width="10.7265625" customWidth="1"/>
-    <col min="10" max="10" width="46.7265625" customWidth="1"/>
-    <col min="11" max="11" width="37.81640625" customWidth="1"/>
-    <col min="12" max="12" width="67.26953125" customWidth="1"/>
+    <col min="8" max="8" width="23.42578125" customWidth="1"/>
+    <col min="9" max="9" width="10.7109375" customWidth="1"/>
+    <col min="10" max="10" width="46.7109375" customWidth="1"/>
+    <col min="11" max="11" width="37.85546875" customWidth="1"/>
+    <col min="12" max="12" width="67.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="27" t="s">
         <v>46</v>
       </c>
@@ -1783,7 +1827,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>58</v>
       </c>
@@ -1818,7 +1862,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>63</v>
       </c>
@@ -1840,7 +1884,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>66</v>
       </c>
@@ -1860,7 +1904,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>68</v>
       </c>
@@ -1880,7 +1924,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>70</v>
       </c>
@@ -1900,7 +1944,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>72</v>
       </c>
@@ -1922,7 +1966,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>75</v>
       </c>
@@ -1942,7 +1986,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>77</v>
       </c>
@@ -1964,7 +2008,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>80</v>
       </c>
@@ -1984,7 +2028,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>82</v>
       </c>
@@ -2007,7 +2051,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
         <v>85</v>
       </c>
@@ -2027,7 +2071,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="29" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>87</v>
       </c>
@@ -2050,7 +2094,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="30" t="s">
         <v>90</v>
       </c>
@@ -2070,7 +2114,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>92</v>
       </c>
@@ -2098,7 +2142,7 @@
       </c>
       <c r="J15" s="41"/>
     </row>
-    <row r="16" spans="1:12" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" ht="285" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
         <v>23</v>
       </c>
@@ -2116,89 +2160,89 @@
       </c>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E17" s="4"/>
       <c r="F17" s="3"/>
       <c r="G17" s="3"/>
       <c r="J17" s="5"/>
     </row>
-    <row r="18" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E18" s="4"/>
       <c r="F18" s="3"/>
       <c r="G18" s="3"/>
       <c r="J18" s="5"/>
     </row>
-    <row r="19" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E19" s="4"/>
       <c r="F19" s="3"/>
       <c r="G19" s="3"/>
       <c r="J19" s="5"/>
     </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E20" s="4"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D21" s="1"/>
       <c r="E21" s="4"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="J21" s="5"/>
     </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E22" s="4"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="J22" s="5"/>
     </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E23" s="2"/>
       <c r="F23" s="3"/>
       <c r="G23" s="3"/>
     </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:10" x14ac:dyDescent="0.25">
       <c r="D24" s="1"/>
       <c r="E24" s="2"/>
       <c r="F24" s="3"/>
       <c r="G24" s="3"/>
     </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E25" s="2"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
     </row>
-    <row r="26" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:10" x14ac:dyDescent="0.25">
       <c r="E26" s="2"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
     </row>
-    <row r="30" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B30" s="11"/>
       <c r="C30" s="6"/>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B31" s="11"/>
       <c r="C31" s="6"/>
     </row>
-    <row r="32" spans="2:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B32" s="11"/>
       <c r="C32" s="6"/>
     </row>
-    <row r="33" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33" s="11"/>
       <c r="C33" s="6"/>
     </row>
-    <row r="34" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34" s="11"/>
       <c r="C34" s="6"/>
     </row>
-    <row r="35" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35" s="11"/>
       <c r="C35" s="6"/>
     </row>
-    <row r="36" spans="2:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="2:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B36" s="14"/>
       <c r="C36" s="15"/>
     </row>

</xml_diff>